<commit_message>
MRPAM: Fill 2022 data gaps in 3 datasets (#102)
Adds 2022 data to mrpam-budget-revenue, mrpam-fuel-prices, and
mrpam-mining-permits. Combined with main's existing 2023-2025 data,
final coverage is now 2022-2025 for all three datasets.

Row counts:
- mrpam-budget-revenue: 248 → 320 (+72 rows for 2022)
- mrpam-fuel-prices: 781 → 1045 (+264 rows for 2022)
- mrpam-mining-permits: 748 → 1012 (+264 rows for 2022)

EN/MN parity verified, all 51/51 dataset checks pass, build green.

Squash-rebased onto current main from original PR commits:
b4f08c0d, 773a220b, cfa37d75.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/mrpam-budget-revenue.xlsx
+++ b/data.mn/public/datasets/mrpam-budget-revenue.xlsx
@@ -28,6 +28,7 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="3">
@@ -39,7 +40,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="002E4057"/>
       </patternFill>
     </fill>
   </fills>
@@ -425,13 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,12 +439,15 @@
         </is>
       </c>
       <c r="B1" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C1" s="1" t="n">
         <v>2023</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="D1" s="1" t="n">
         <v>2024</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="E1" s="1" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -456,11 +457,9 @@
           <t>(Cont.Table 1.5) Mining license Area size Number Share to total Hectare Share to total Construction Rock</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>19024.8</v>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -468,11 +467,9 @@
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>2793.1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -480,11 +477,9 @@
           <t>Bazalit</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>1370.9</v>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -492,11 +487,9 @@
           <t>Bitumen</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>601.5</v>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -504,11 +497,9 @@
           <t>Common Construction</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>599.1</v>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -516,11 +507,9 @@
           <t>Common mineral</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>183.5</v>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -528,11 +517,9 @@
           <t>Concentrated metal</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>4533.3</v>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -540,11 +527,9 @@
           <t>Construction materials</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>2009.2</v>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -552,11 +537,9 @@
           <t>Copper</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>21148.8</v>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -564,11 +547,9 @@
           <t>Face stone</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>2618.6</v>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -576,11 +557,9 @@
           <t>Glauberic salt</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>1449</v>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -588,11 +567,9 @@
           <t>Gold</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>16385.5</v>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -600,11 +577,9 @@
           <t>Gold (placer)</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>33619.7</v>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -612,11 +587,9 @@
           <t>Gold ore</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>6206</v>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -624,11 +597,9 @@
           <t>Gold оre</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>4668.6</v>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -636,11 +607,9 @@
           <t>Granite</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="C17" t="n">
         <v>275.3</v>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -648,11 +617,9 @@
           <t>Graphite</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>3000.6</v>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -660,11 +627,9 @@
           <t>Iron</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>5593.9</v>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -672,11 +637,9 @@
           <t>Keramzite Clay</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>207.8</v>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -684,11 +647,9 @@
           <t>Lithium</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>4720.2</v>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -696,9 +657,7 @@
           <t>Mining license fee</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>273678</v>
       </c>
     </row>
@@ -708,9 +667,7 @@
           <t>Other revenue</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>24677.8</v>
       </c>
     </row>
@@ -720,11 +677,9 @@
           <t>Perlit</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="C24" t="n">
         <v>771.5</v>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -732,9 +687,7 @@
           <t>Petroleum export revenue</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
         <v>1560266.3</v>
       </c>
     </row>
@@ -744,11 +697,9 @@
           <t>Precious stones</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="C26" t="n">
         <v>593.2</v>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -756,11 +707,9 @@
           <t>Quartz</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="C27" t="n">
         <v>525.4</v>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -768,9 +717,7 @@
           <t>Reimbursement for state-funded exploration</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="n">
+      <c r="E28" t="n">
         <v>16033.5</v>
       </c>
     </row>
@@ -780,11 +727,9 @@
           <t>Sand</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="C29" t="n">
         <v>21927.3</v>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -792,11 +737,9 @@
           <t>Silicium</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="C30" t="n">
         <v>9587.700000000001</v>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -804,11 +747,9 @@
           <t>Silver</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="C31" t="n">
         <v>1050.4</v>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -816,9 +757,7 @@
           <t>Tender revenue</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="n">
+      <c r="E32" t="n">
         <v>674535.2</v>
       </c>
     </row>
@@ -828,9 +767,7 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="n">
+      <c r="E33" t="n">
         <v>2549190.8</v>
       </c>
     </row>
@@ -840,11 +777,9 @@
           <t>Tungsten</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="C34" t="n">
         <v>2833.9</v>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -852,11 +787,9 @@
           <t>Zinc</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="C35" t="n">
         <v>1969.8</v>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -864,13 +797,12 @@
           <t>Ашигт малтмалын тусгай зөвшөөрлийн төлбөр</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="C36" t="n">
         <v>199646.1</v>
       </c>
-      <c r="C36" t="n">
+      <c r="D36" t="n">
         <v>245388.4</v>
       </c>
-      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -878,13 +810,12 @@
           <t>Бусад орлого</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="C37" t="n">
         <v>35777.2</v>
       </c>
-      <c r="C37" t="n">
+      <c r="D37" t="n">
         <v>23028</v>
       </c>
-      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -892,13 +823,12 @@
           <t>БҮГД</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="C38" t="n">
         <v>2126263.2</v>
       </c>
-      <c r="C38" t="n">
+      <c r="D38" t="n">
         <v>2121407.8</v>
       </c>
-      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -906,13 +836,12 @@
           <t>Газрын тосны экспорт</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="C39" t="n">
         <v>1601164.4</v>
       </c>
-      <c r="C39" t="n">
+      <c r="D39" t="n">
         <v>1498017.5</v>
       </c>
-      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -920,13 +849,12 @@
           <t>Сонгон шалгаруулалт</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="C40" t="n">
         <v>279981.9</v>
       </c>
-      <c r="C40" t="n">
+      <c r="D40" t="n">
         <v>338645.5</v>
       </c>
-      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -934,13 +862,12 @@
           <t>Улсын төсвийн хөрөнгөөр хайгуул хийсэн ордын нөхөн төлбөр</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="C41" t="n">
         <v>9693.799999999999</v>
       </c>
-      <c r="C41" t="n">
+      <c r="D41" t="n">
         <v>16328.4</v>
       </c>
-      <c r="D41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -953,13 +880,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -969,12 +893,15 @@
         </is>
       </c>
       <c r="B1" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C1" s="1" t="n">
         <v>2023</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="D1" s="1" t="n">
         <v>2024</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="E1" s="1" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -984,11 +911,9 @@
           <t>(Cont.Table 1.5) Mining license Area size Number Share to total Hectare Share to total Construction Rock</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>19024.8</v>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -996,11 +921,9 @@
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>2793.1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1008,11 +931,9 @@
           <t>Bazalit</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>1370.9</v>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1020,11 +941,9 @@
           <t>Bitumen</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>601.5</v>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1032,11 +951,9 @@
           <t>Common Construction</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>599.1</v>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1044,11 +961,9 @@
           <t>Common mineral</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>183.5</v>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1056,11 +971,9 @@
           <t>Concentrated metal</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>4533.3</v>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1068,11 +981,9 @@
           <t>Construction materials</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>2009.2</v>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1080,11 +991,9 @@
           <t>Copper</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>21148.8</v>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1092,11 +1001,9 @@
           <t>Face stone</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>2618.6</v>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1104,11 +1011,9 @@
           <t>Glauberic salt</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>1449</v>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1116,11 +1021,9 @@
           <t>Gold</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>16385.5</v>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1128,11 +1031,9 @@
           <t>Gold (placer)</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>33619.7</v>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1140,11 +1041,9 @@
           <t>Gold ore</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>6206</v>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1152,11 +1051,9 @@
           <t>Gold оre</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>4668.6</v>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1164,11 +1061,9 @@
           <t>Granite</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="C17" t="n">
         <v>275.3</v>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1176,11 +1071,9 @@
           <t>Graphite</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>3000.6</v>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1188,11 +1081,9 @@
           <t>Iron</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>5593.9</v>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1200,11 +1091,9 @@
           <t>Keramzite Clay</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>207.8</v>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1212,11 +1101,9 @@
           <t>Lithium</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>4720.2</v>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1224,11 +1111,9 @@
           <t>Perlit</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="C22" t="n">
         <v>771.5</v>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1236,11 +1121,9 @@
           <t>Precious stones</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="C23" t="n">
         <v>593.2</v>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1248,11 +1131,9 @@
           <t>Quartz</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="C24" t="n">
         <v>525.4</v>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1260,11 +1141,9 @@
           <t>Sand</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="C25" t="n">
         <v>21927.3</v>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1272,11 +1151,9 @@
           <t>Silicium</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="C26" t="n">
         <v>9587.700000000001</v>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1284,11 +1161,9 @@
           <t>Silver</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="C27" t="n">
         <v>1050.4</v>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1296,11 +1171,9 @@
           <t>Tungsten</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="C28" t="n">
         <v>2833.9</v>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1308,11 +1181,9 @@
           <t>Zinc</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="C29" t="n">
         <v>1969.8</v>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1321,12 +1192,15 @@
         </is>
       </c>
       <c r="B30" t="n">
+        <v>217812.4</v>
+      </c>
+      <c r="C30" t="n">
         <v>199646.1</v>
       </c>
-      <c r="C30" t="n">
+      <c r="D30" t="n">
         <v>245388.4</v>
       </c>
-      <c r="D30" t="n">
+      <c r="E30" t="n">
         <v>273678</v>
       </c>
     </row>
@@ -1337,12 +1211,15 @@
         </is>
       </c>
       <c r="B31" t="n">
+        <v>29460.5</v>
+      </c>
+      <c r="C31" t="n">
         <v>35777.2</v>
       </c>
-      <c r="C31" t="n">
+      <c r="D31" t="n">
         <v>23028</v>
       </c>
-      <c r="D31" t="n">
+      <c r="E31" t="n">
         <v>24677.8</v>
       </c>
     </row>
@@ -1353,12 +1230,15 @@
         </is>
       </c>
       <c r="B32" t="n">
+        <v>922249.6</v>
+      </c>
+      <c r="C32" t="n">
         <v>2126263.2</v>
       </c>
-      <c r="C32" t="n">
+      <c r="D32" t="n">
         <v>2121407.8</v>
       </c>
-      <c r="D32" t="n">
+      <c r="E32" t="n">
         <v>2549190.8</v>
       </c>
     </row>
@@ -1369,12 +1249,15 @@
         </is>
       </c>
       <c r="B33" t="n">
+        <v>510992.9</v>
+      </c>
+      <c r="C33" t="n">
         <v>1601164.4</v>
       </c>
-      <c r="C33" t="n">
+      <c r="D33" t="n">
         <v>1498017.5</v>
       </c>
-      <c r="D33" t="n">
+      <c r="E33" t="n">
         <v>1560266.3</v>
       </c>
     </row>
@@ -1385,12 +1268,15 @@
         </is>
       </c>
       <c r="B34" t="n">
+        <v>155030.6</v>
+      </c>
+      <c r="C34" t="n">
         <v>279981.9</v>
       </c>
-      <c r="C34" t="n">
+      <c r="D34" t="n">
         <v>338645.5</v>
       </c>
-      <c r="D34" t="n">
+      <c r="E34" t="n">
         <v>674535.2</v>
       </c>
     </row>
@@ -1400,14 +1286,24 @@
           <t>Улсын төсвийн хөрөнгөөр хайгуул хийсэн ордын нөхөн төлбөр</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="C35" t="n">
         <v>9693.799999999999</v>
       </c>
-      <c r="C35" t="n">
+      <c r="D35" t="n">
         <v>16328.4</v>
       </c>
-      <c r="D35" t="n">
+      <c r="E35" t="n">
         <v>16033.5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Хайгуулын ордын нөхөн төлбөр</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>8953.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>